<commit_message>
Add generic field detection for login automation
</commit_message>
<xml_diff>
--- a/accounts.xlsx
+++ b/accounts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gowri\New folder (9)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5691A51-DD9D-4F15-A769-F019FBE3A9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F614F226-D233-4D1D-B7FC-DA37A83DEB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>URL</t>
   </si>
@@ -31,13 +31,22 @@
     <t>Password</t>
   </si>
   <si>
-    <t>https://the-internet.herokuapp.com/login</t>
-  </si>
-  <si>
-    <t>tomsmith</t>
-  </si>
-  <si>
-    <t>SuperSecretPassword!</t>
+    <t>https://practicetestautomation.com/practice-test-login/</t>
+  </si>
+  <si>
+    <t>student</t>
+  </si>
+  <si>
+    <t>Password123</t>
+  </si>
+  <si>
+    <t>Bia@5836</t>
+  </si>
+  <si>
+    <t>https://vjcet.etlab.in/user/login</t>
+  </si>
+  <si>
+    <t>23rr176</t>
   </si>
 </sst>
 </file>
@@ -402,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -422,18 +431,34 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{2503EDB8-6D2A-4872-B1F1-5E688CBC736B}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{D7B2C6BF-D95F-425E-97E7-01463A669578}"/>
+    <hyperlink ref="A2" r:id="rId2" xr:uid="{2503EDB8-6D2A-4872-B1F1-5E688CBC736B}"/>
+    <hyperlink ref="C2" r:id="rId3" xr:uid="{74C2FD94-1F3D-4869-9723-4E70E2BE28A0}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>